<commit_message>
Review 10 Problems 2/23/2026
</commit_message>
<xml_diff>
--- a/Code & Notes/Functions & Notes.xlsx
+++ b/Code & Notes/Functions & Notes.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="23127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\My Career\Courses\Web Development\Problem Solving\Code &amp; Notes\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F91DA777-0C1A-4DC7-AE3D-C088F09C8C72}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{66C2B70E-C977-4F92-A030-E6EC68BA5C6D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -794,6 +794,24 @@
     <xf numFmtId="0" fontId="4" fillId="23" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="21" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="22" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="15" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -806,9 +824,6 @@
     <xf numFmtId="0" fontId="3" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -832,21 +847,6 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="21" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="22" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1150,10 +1150,10 @@
       </c>
     </row>
     <row r="2" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
-      <c r="A2" s="41" t="s">
+      <c r="A2" s="47" t="s">
         <v>81</v>
       </c>
-      <c r="B2" s="41"/>
+      <c r="B2" s="47"/>
     </row>
     <row r="3" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
@@ -1172,10 +1172,10 @@
       </c>
     </row>
     <row r="5" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A5" s="46" t="s">
+      <c r="A5" s="51" t="s">
         <v>78</v>
       </c>
-      <c r="B5" s="46"/>
+      <c r="B5" s="51"/>
     </row>
     <row r="6" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A6" s="4" t="s">
@@ -1226,10 +1226,10 @@
       </c>
     </row>
     <row r="12" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A12" s="47" t="s">
+      <c r="A12" s="52" t="s">
         <v>79</v>
       </c>
-      <c r="B12" s="47"/>
+      <c r="B12" s="52"/>
     </row>
     <row r="13" spans="1:2" ht="29" x14ac:dyDescent="0.35">
       <c r="A13" s="7" t="s">
@@ -1240,10 +1240,10 @@
       </c>
     </row>
     <row r="14" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A14" s="48" t="s">
+      <c r="A14" s="53" t="s">
         <v>80</v>
       </c>
-      <c r="B14" s="48"/>
+      <c r="B14" s="53"/>
     </row>
     <row r="15" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A15" s="9" t="s">
@@ -1262,10 +1262,10 @@
       </c>
     </row>
     <row r="17" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A17" s="42" t="s">
+      <c r="A17" s="48" t="s">
         <v>82</v>
       </c>
-      <c r="B17" s="42"/>
+      <c r="B17" s="48"/>
     </row>
     <row r="18" spans="1:2" s="1" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A18" s="11" t="s">
@@ -1316,10 +1316,10 @@
       </c>
     </row>
     <row r="24" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A24" s="49" t="s">
+      <c r="A24" s="54" t="s">
         <v>85</v>
       </c>
-      <c r="B24" s="49"/>
+      <c r="B24" s="54"/>
     </row>
     <row r="25" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A25" s="27" t="s">
@@ -1354,10 +1354,10 @@
       </c>
     </row>
     <row r="29" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A29" s="50" t="s">
+      <c r="A29" s="55" t="s">
         <v>86</v>
       </c>
-      <c r="B29" s="50"/>
+      <c r="B29" s="55"/>
     </row>
     <row r="30" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A30" s="17" t="s">
@@ -1376,10 +1376,10 @@
       </c>
     </row>
     <row r="32" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A32" s="51" t="s">
+      <c r="A32" s="56" t="s">
         <v>87</v>
       </c>
-      <c r="B32" s="51"/>
+      <c r="B32" s="56"/>
     </row>
     <row r="33" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A33" s="19" t="s">
@@ -1422,10 +1422,10 @@
       </c>
     </row>
     <row r="38" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A38" s="52" t="s">
+      <c r="A38" s="57" t="s">
         <v>89</v>
       </c>
-      <c r="B38" s="52"/>
+      <c r="B38" s="57"/>
     </row>
     <row r="39" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A39" s="24" t="s">
@@ -1444,10 +1444,10 @@
       </c>
     </row>
     <row r="41" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
-      <c r="A41" s="53" t="s">
+      <c r="A41" s="58" t="s">
         <v>91</v>
       </c>
-      <c r="B41" s="53"/>
+      <c r="B41" s="58"/>
     </row>
     <row r="42" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A42" s="29" t="s">
@@ -1482,16 +1482,16 @@
       </c>
     </row>
     <row r="46" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A46" s="43" t="s">
+      <c r="A46" s="49" t="s">
         <v>43</v>
       </c>
-      <c r="B46" s="45" t="s">
+      <c r="B46" s="43" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="47" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A47" s="44"/>
-      <c r="B47" s="45"/>
+      <c r="A47" s="50"/>
+      <c r="B47" s="43"/>
     </row>
     <row r="48" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A48" s="31" t="s">
@@ -1534,24 +1534,24 @@
       </c>
     </row>
     <row r="53" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A53" s="54" t="s">
+      <c r="A53" s="41" t="s">
         <v>94</v>
       </c>
-      <c r="B53" s="45" t="s">
+      <c r="B53" s="43" t="s">
         <v>95</v>
       </c>
     </row>
     <row r="54" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A54" s="55"/>
-      <c r="B54" s="45"/>
+      <c r="A54" s="42"/>
+      <c r="B54" s="43"/>
     </row>
     <row r="55" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A55" s="55"/>
-      <c r="B55" s="45"/>
+      <c r="A55" s="42"/>
+      <c r="B55" s="43"/>
     </row>
     <row r="56" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A56" s="55"/>
-      <c r="B56" s="45"/>
+      <c r="A56" s="42"/>
+      <c r="B56" s="43"/>
     </row>
     <row r="57" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A57" s="31" t="s">
@@ -1586,10 +1586,10 @@
       </c>
     </row>
     <row r="61" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A61" s="56" t="s">
+      <c r="A61" s="44" t="s">
         <v>93</v>
       </c>
-      <c r="B61" s="56"/>
+      <c r="B61" s="44"/>
     </row>
     <row r="62" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A62" s="32" t="s">
@@ -1648,10 +1648,10 @@
       </c>
     </row>
     <row r="69" spans="1:2" ht="18.5" x14ac:dyDescent="0.35">
-      <c r="A69" s="58" t="s">
+      <c r="A69" s="46" t="s">
         <v>88</v>
       </c>
-      <c r="B69" s="58"/>
+      <c r="B69" s="46"/>
     </row>
     <row r="70" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A70" s="21" t="s">
@@ -1742,10 +1742,10 @@
       </c>
     </row>
     <row r="81" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
-      <c r="A81" s="57" t="s">
+      <c r="A81" s="45" t="s">
         <v>127</v>
       </c>
-      <c r="B81" s="57"/>
+      <c r="B81" s="45"/>
     </row>
     <row r="82" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A82" s="39" t="s">
@@ -1765,11 +1765,6 @@
     </row>
   </sheetData>
   <mergeCells count="17">
-    <mergeCell ref="A53:A56"/>
-    <mergeCell ref="B53:B56"/>
-    <mergeCell ref="A61:B61"/>
-    <mergeCell ref="A81:B81"/>
-    <mergeCell ref="A69:B69"/>
     <mergeCell ref="A2:B2"/>
     <mergeCell ref="A17:B17"/>
     <mergeCell ref="A46:A47"/>
@@ -1782,6 +1777,11 @@
     <mergeCell ref="A32:B32"/>
     <mergeCell ref="A38:B38"/>
     <mergeCell ref="A41:B41"/>
+    <mergeCell ref="A53:A56"/>
+    <mergeCell ref="B53:B56"/>
+    <mergeCell ref="A61:B61"/>
+    <mergeCell ref="A81:B81"/>
+    <mergeCell ref="A69:B69"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
Reviewed 3 Problems 5/10/2026
</commit_message>
<xml_diff>
--- a/Code & Notes/Functions & Notes.xlsx
+++ b/Code & Notes/Functions & Notes.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\My Career\Courses\Web Development\Problem Solving\Code &amp; Notes\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{66C2B70E-C977-4F92-A030-E6EC68BA5C6D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{77EA04D4-49F6-4426-9076-152114C25267}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -794,15 +794,51 @@
     <xf numFmtId="0" fontId="4" fillId="23" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="15" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="16" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="17" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="18" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="19" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="21" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -811,42 +847,6 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="15" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="16" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="17" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="18" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="19" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1150,10 +1150,10 @@
       </c>
     </row>
     <row r="2" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
-      <c r="A2" s="47" t="s">
+      <c r="A2" s="41" t="s">
         <v>81</v>
       </c>
-      <c r="B2" s="47"/>
+      <c r="B2" s="41"/>
     </row>
     <row r="3" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
@@ -1172,10 +1172,10 @@
       </c>
     </row>
     <row r="5" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A5" s="51" t="s">
+      <c r="A5" s="46" t="s">
         <v>78</v>
       </c>
-      <c r="B5" s="51"/>
+      <c r="B5" s="46"/>
     </row>
     <row r="6" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A6" s="4" t="s">
@@ -1226,10 +1226,10 @@
       </c>
     </row>
     <row r="12" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A12" s="52" t="s">
+      <c r="A12" s="47" t="s">
         <v>79</v>
       </c>
-      <c r="B12" s="52"/>
+      <c r="B12" s="47"/>
     </row>
     <row r="13" spans="1:2" ht="29" x14ac:dyDescent="0.35">
       <c r="A13" s="7" t="s">
@@ -1240,10 +1240,10 @@
       </c>
     </row>
     <row r="14" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A14" s="53" t="s">
+      <c r="A14" s="48" t="s">
         <v>80</v>
       </c>
-      <c r="B14" s="53"/>
+      <c r="B14" s="48"/>
     </row>
     <row r="15" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A15" s="9" t="s">
@@ -1262,10 +1262,10 @@
       </c>
     </row>
     <row r="17" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A17" s="48" t="s">
+      <c r="A17" s="42" t="s">
         <v>82</v>
       </c>
-      <c r="B17" s="48"/>
+      <c r="B17" s="42"/>
     </row>
     <row r="18" spans="1:2" s="1" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A18" s="11" t="s">
@@ -1316,10 +1316,10 @@
       </c>
     </row>
     <row r="24" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A24" s="54" t="s">
+      <c r="A24" s="49" t="s">
         <v>85</v>
       </c>
-      <c r="B24" s="54"/>
+      <c r="B24" s="49"/>
     </row>
     <row r="25" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A25" s="27" t="s">
@@ -1354,10 +1354,10 @@
       </c>
     </row>
     <row r="29" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A29" s="55" t="s">
+      <c r="A29" s="50" t="s">
         <v>86</v>
       </c>
-      <c r="B29" s="55"/>
+      <c r="B29" s="50"/>
     </row>
     <row r="30" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A30" s="17" t="s">
@@ -1376,10 +1376,10 @@
       </c>
     </row>
     <row r="32" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A32" s="56" t="s">
+      <c r="A32" s="51" t="s">
         <v>87</v>
       </c>
-      <c r="B32" s="56"/>
+      <c r="B32" s="51"/>
     </row>
     <row r="33" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A33" s="19" t="s">
@@ -1422,10 +1422,10 @@
       </c>
     </row>
     <row r="38" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A38" s="57" t="s">
+      <c r="A38" s="52" t="s">
         <v>89</v>
       </c>
-      <c r="B38" s="57"/>
+      <c r="B38" s="52"/>
     </row>
     <row r="39" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A39" s="24" t="s">
@@ -1444,10 +1444,10 @@
       </c>
     </row>
     <row r="41" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
-      <c r="A41" s="58" t="s">
+      <c r="A41" s="53" t="s">
         <v>91</v>
       </c>
-      <c r="B41" s="58"/>
+      <c r="B41" s="53"/>
     </row>
     <row r="42" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A42" s="29" t="s">
@@ -1482,16 +1482,16 @@
       </c>
     </row>
     <row r="46" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A46" s="49" t="s">
+      <c r="A46" s="43" t="s">
         <v>43</v>
       </c>
-      <c r="B46" s="43" t="s">
+      <c r="B46" s="45" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="47" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A47" s="50"/>
-      <c r="B47" s="43"/>
+      <c r="A47" s="44"/>
+      <c r="B47" s="45"/>
     </row>
     <row r="48" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A48" s="31" t="s">
@@ -1534,24 +1534,24 @@
       </c>
     </row>
     <row r="53" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A53" s="41" t="s">
+      <c r="A53" s="54" t="s">
         <v>94</v>
       </c>
-      <c r="B53" s="43" t="s">
+      <c r="B53" s="45" t="s">
         <v>95</v>
       </c>
     </row>
     <row r="54" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A54" s="42"/>
-      <c r="B54" s="43"/>
+      <c r="A54" s="55"/>
+      <c r="B54" s="45"/>
     </row>
     <row r="55" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A55" s="42"/>
-      <c r="B55" s="43"/>
+      <c r="A55" s="55"/>
+      <c r="B55" s="45"/>
     </row>
     <row r="56" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A56" s="42"/>
-      <c r="B56" s="43"/>
+      <c r="A56" s="55"/>
+      <c r="B56" s="45"/>
     </row>
     <row r="57" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A57" s="31" t="s">
@@ -1586,10 +1586,10 @@
       </c>
     </row>
     <row r="61" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A61" s="44" t="s">
+      <c r="A61" s="56" t="s">
         <v>93</v>
       </c>
-      <c r="B61" s="44"/>
+      <c r="B61" s="56"/>
     </row>
     <row r="62" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A62" s="32" t="s">
@@ -1648,10 +1648,10 @@
       </c>
     </row>
     <row r="69" spans="1:2" ht="18.5" x14ac:dyDescent="0.35">
-      <c r="A69" s="46" t="s">
+      <c r="A69" s="58" t="s">
         <v>88</v>
       </c>
-      <c r="B69" s="46"/>
+      <c r="B69" s="58"/>
     </row>
     <row r="70" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A70" s="21" t="s">
@@ -1742,10 +1742,10 @@
       </c>
     </row>
     <row r="81" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
-      <c r="A81" s="45" t="s">
+      <c r="A81" s="57" t="s">
         <v>127</v>
       </c>
-      <c r="B81" s="45"/>
+      <c r="B81" s="57"/>
     </row>
     <row r="82" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A82" s="39" t="s">
@@ -1765,6 +1765,11 @@
     </row>
   </sheetData>
   <mergeCells count="17">
+    <mergeCell ref="A53:A56"/>
+    <mergeCell ref="B53:B56"/>
+    <mergeCell ref="A61:B61"/>
+    <mergeCell ref="A81:B81"/>
+    <mergeCell ref="A69:B69"/>
     <mergeCell ref="A2:B2"/>
     <mergeCell ref="A17:B17"/>
     <mergeCell ref="A46:A47"/>
@@ -1777,11 +1782,6 @@
     <mergeCell ref="A32:B32"/>
     <mergeCell ref="A38:B38"/>
     <mergeCell ref="A41:B41"/>
-    <mergeCell ref="A53:A56"/>
-    <mergeCell ref="B53:B56"/>
-    <mergeCell ref="A61:B61"/>
-    <mergeCell ref="A81:B81"/>
-    <mergeCell ref="A69:B69"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
Reviewed 9 Problems 5/13/2026
</commit_message>
<xml_diff>
--- a/Code & Notes/Functions & Notes.xlsx
+++ b/Code & Notes/Functions & Notes.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\My Career\Courses\Web Development\Problem Solving\Code &amp; Notes\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A041B202-C0AE-4C4A-8707-08843D53FADE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C71BCF41-715F-4317-959F-6CA5E5304634}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="120">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="122" uniqueCount="118">
   <si>
     <t>Description</t>
   </si>
@@ -215,9 +215,6 @@
   </si>
   <si>
     <t>remove space in middle from string</t>
-  </si>
-  <si>
-    <t>Let numbers = s.match(/\d+/g);</t>
   </si>
   <si>
     <t>String To Number Or Number To String</t>
@@ -325,9 +322,6 @@
   </si>
   <si>
     <t>remove Numbers away And Return String</t>
-  </si>
-  <si>
-    <t>Return Stringed Numbers From String</t>
   </si>
   <si>
     <t>num.toString(16)</t>
@@ -685,15 +679,42 @@
     <xf numFmtId="0" fontId="4" fillId="19" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="15" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="17" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -702,33 +723,6 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="15" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1025,17 +1019,17 @@
   <sheetData>
     <row r="1" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A1" s="21" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B1" s="21" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="2" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A2" s="43" t="s">
-        <v>64</v>
-      </c>
-      <c r="B2" s="43"/>
+      <c r="A2" s="38" t="s">
+        <v>63</v>
+      </c>
+      <c r="B2" s="38"/>
     </row>
     <row r="3" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
@@ -1054,10 +1048,10 @@
       </c>
     </row>
     <row r="5" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A5" s="40" t="s">
-        <v>65</v>
-      </c>
-      <c r="B5" s="40"/>
+      <c r="A5" s="34" t="s">
+        <v>64</v>
+      </c>
+      <c r="B5" s="34"/>
     </row>
     <row r="6" spans="1:2" s="1" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A6" s="4" t="s">
@@ -1088,7 +1082,7 @@
         <v>36</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="10" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
@@ -1101,17 +1095,17 @@
     </row>
     <row r="11" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A11" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="B11" s="5" t="s">
         <v>87</v>
       </c>
-      <c r="B11" s="5" t="s">
-        <v>88</v>
-      </c>
     </row>
     <row r="12" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A12" s="44" t="s">
-        <v>68</v>
-      </c>
-      <c r="B12" s="44"/>
+      <c r="A12" s="39" t="s">
+        <v>67</v>
+      </c>
+      <c r="B12" s="39"/>
     </row>
     <row r="13" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A13" s="20" t="s">
@@ -1146,10 +1140,10 @@
       </c>
     </row>
     <row r="17" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A17" s="45" t="s">
-        <v>69</v>
-      </c>
-      <c r="B17" s="45"/>
+      <c r="A17" s="40" t="s">
+        <v>68</v>
+      </c>
+      <c r="B17" s="40"/>
     </row>
     <row r="18" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A18" s="10" t="s">
@@ -1168,10 +1162,10 @@
       </c>
     </row>
     <row r="20" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A20" s="46" t="s">
-        <v>70</v>
-      </c>
-      <c r="B20" s="46"/>
+      <c r="A20" s="41" t="s">
+        <v>69</v>
+      </c>
+      <c r="B20" s="41"/>
     </row>
     <row r="21" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A21" s="12" t="s">
@@ -1207,17 +1201,17 @@
     </row>
     <row r="25" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A25" s="12" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="B25" s="28" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
     </row>
     <row r="26" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A26" s="47" t="s">
-        <v>72</v>
-      </c>
-      <c r="B26" s="47"/>
+      <c r="A26" s="42" t="s">
+        <v>71</v>
+      </c>
+      <c r="B26" s="42"/>
     </row>
     <row r="27" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A27" s="17" t="s">
@@ -1236,10 +1230,10 @@
       </c>
     </row>
     <row r="29" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
-      <c r="A29" s="48" t="s">
-        <v>74</v>
-      </c>
-      <c r="B29" s="48"/>
+      <c r="A29" s="43" t="s">
+        <v>73</v>
+      </c>
+      <c r="B29" s="43"/>
     </row>
     <row r="30" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A30" s="22" t="s">
@@ -1251,10 +1245,10 @@
     </row>
     <row r="31" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A31" s="23" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="B31" s="23" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
     </row>
     <row r="32" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
@@ -1274,16 +1268,16 @@
       </c>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A34" s="41" t="s">
+      <c r="A34" s="35" t="s">
         <v>31</v>
       </c>
-      <c r="B34" s="36" t="s">
+      <c r="B34" s="37" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A35" s="42"/>
-      <c r="B35" s="36"/>
+      <c r="A35" s="36"/>
+      <c r="B35" s="37"/>
     </row>
     <row r="36" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A36" s="24" t="s">
@@ -1295,7 +1289,7 @@
     </row>
     <row r="37" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A37" s="24" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="B37" s="23" t="s">
         <v>43</v>
@@ -1303,7 +1297,7 @@
     </row>
     <row r="38" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A38" s="24" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B38" s="23" t="s">
         <v>44</v>
@@ -1326,69 +1320,69 @@
       </c>
     </row>
     <row r="41" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A41" s="34" t="s">
+      <c r="A41" s="44" t="s">
+        <v>76</v>
+      </c>
+      <c r="B41" s="37" t="s">
         <v>77</v>
       </c>
-      <c r="B41" s="36" t="s">
-        <v>78</v>
-      </c>
     </row>
     <row r="42" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A42" s="35"/>
-      <c r="B42" s="36"/>
+      <c r="A42" s="45"/>
+      <c r="B42" s="37"/>
     </row>
     <row r="43" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A43" s="35"/>
-      <c r="B43" s="36"/>
+      <c r="A43" s="45"/>
+      <c r="B43" s="37"/>
     </row>
     <row r="44" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A44" s="35"/>
-      <c r="B44" s="36"/>
+      <c r="A44" s="45"/>
+      <c r="B44" s="37"/>
     </row>
     <row r="45" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A45" s="24" t="s">
+        <v>78</v>
+      </c>
+      <c r="B45" s="22" t="s">
         <v>79</v>
-      </c>
-      <c r="B45" s="22" t="s">
-        <v>80</v>
       </c>
     </row>
     <row r="46" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A46" s="24" t="s">
+        <v>80</v>
+      </c>
+      <c r="B46" s="22" t="s">
         <v>81</v>
-      </c>
-      <c r="B46" s="22" t="s">
-        <v>82</v>
       </c>
     </row>
     <row r="47" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A47" s="24" t="s">
+        <v>94</v>
+      </c>
+      <c r="B47" s="22" t="s">
         <v>95</v>
-      </c>
-      <c r="B47" s="22" t="s">
-        <v>96</v>
       </c>
     </row>
     <row r="48" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A48" s="24" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="B48" s="22" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
     </row>
     <row r="49" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A49" s="37" t="s">
-        <v>76</v>
-      </c>
-      <c r="B49" s="37"/>
+      <c r="A49" s="46" t="s">
+        <v>75</v>
+      </c>
+      <c r="B49" s="46"/>
     </row>
     <row r="50" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A50" s="25" t="s">
         <v>49</v>
       </c>
       <c r="B50" s="26" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="51" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
@@ -1401,49 +1395,49 @@
     </row>
     <row r="52" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A52" s="25" t="s">
+        <v>65</v>
+      </c>
+      <c r="B52" s="26" t="s">
         <v>66</v>
-      </c>
-      <c r="B52" s="26" t="s">
-        <v>67</v>
       </c>
     </row>
     <row r="53" spans="1:2" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A53" s="29" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B53" s="30" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
     </row>
     <row r="54" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A54" s="29" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="B54" s="30" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
     </row>
     <row r="55" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A55" s="29" t="s">
+        <v>91</v>
+      </c>
+      <c r="B55" s="30" t="s">
         <v>92</v>
-      </c>
-      <c r="B55" s="30" t="s">
-        <v>93</v>
       </c>
     </row>
     <row r="56" spans="1:2" ht="29" x14ac:dyDescent="0.35">
       <c r="A56" s="29" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="B56" s="30" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
     </row>
     <row r="57" spans="1:2" ht="18.5" x14ac:dyDescent="0.35">
-      <c r="A57" s="39" t="s">
-        <v>71</v>
-      </c>
-      <c r="B57" s="39"/>
+      <c r="A57" s="48" t="s">
+        <v>70</v>
+      </c>
+      <c r="B57" s="48"/>
     </row>
     <row r="58" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A58" s="14" t="s">
@@ -1458,7 +1452,7 @@
         <v>33</v>
       </c>
       <c r="B59" s="15" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="60" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
@@ -1470,19 +1464,15 @@
       </c>
     </row>
     <row r="61" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A61" s="14" t="s">
-        <v>63</v>
-      </c>
-      <c r="B61" s="15" t="s">
-        <v>98</v>
-      </c>
+      <c r="A61" s="14"/>
+      <c r="B61" s="15"/>
     </row>
     <row r="62" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A62" s="16" t="s">
         <v>56</v>
       </c>
       <c r="B62" s="15" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
     <row r="63" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
@@ -1495,68 +1485,73 @@
     </row>
     <row r="64" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A64" s="16" t="s">
+        <v>82</v>
+      </c>
+      <c r="B64" s="15" t="s">
         <v>83</v>
-      </c>
-      <c r="B64" s="15" t="s">
-        <v>84</v>
       </c>
     </row>
     <row r="65" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A65" s="16" t="s">
+        <v>88</v>
+      </c>
+      <c r="B65" s="15" t="s">
         <v>89</v>
-      </c>
-      <c r="B65" s="15" t="s">
-        <v>90</v>
       </c>
     </row>
     <row r="66" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A66" s="31" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="B66" s="15" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
     </row>
     <row r="67" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A67" s="16" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="B67" s="15" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
     </row>
     <row r="68" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A68" s="16" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="B68" s="15" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
     </row>
     <row r="69" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
-      <c r="A69" s="38" t="s">
-        <v>110</v>
-      </c>
-      <c r="B69" s="38"/>
+      <c r="A69" s="47" t="s">
+        <v>108</v>
+      </c>
+      <c r="B69" s="47"/>
     </row>
     <row r="70" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A70" s="32" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="B70" s="33" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
     </row>
     <row r="71" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A71" s="32" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="B71" s="33" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="14">
+    <mergeCell ref="A41:A44"/>
+    <mergeCell ref="B41:B44"/>
+    <mergeCell ref="A49:B49"/>
+    <mergeCell ref="A69:B69"/>
+    <mergeCell ref="A57:B57"/>
     <mergeCell ref="A5:B5"/>
     <mergeCell ref="A34:A35"/>
     <mergeCell ref="B34:B35"/>
@@ -1566,11 +1561,6 @@
     <mergeCell ref="A20:B20"/>
     <mergeCell ref="A26:B26"/>
     <mergeCell ref="A29:B29"/>
-    <mergeCell ref="A41:A44"/>
-    <mergeCell ref="B41:B44"/>
-    <mergeCell ref="A49:B49"/>
-    <mergeCell ref="A69:B69"/>
-    <mergeCell ref="A57:B57"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
Reviewed 5 Problems 5/14/2026
</commit_message>
<xml_diff>
--- a/Code & Notes/Functions & Notes.xlsx
+++ b/Code & Notes/Functions & Notes.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\My Career\Courses\Web Development\Problem Solving\Code &amp; Notes\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C71BCF41-715F-4317-959F-6CA5E5304634}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A6CE14E-42F3-4544-BA4C-E82C0969CC24}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -679,6 +679,24 @@
     <xf numFmtId="0" fontId="4" fillId="19" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="17" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="18" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -688,9 +706,6 @@
     <xf numFmtId="0" fontId="3" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
@@ -708,21 +723,6 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="17" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="18" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1026,10 +1026,10 @@
       </c>
     </row>
     <row r="2" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A2" s="38" t="s">
+      <c r="A2" s="43" t="s">
         <v>63</v>
       </c>
-      <c r="B2" s="38"/>
+      <c r="B2" s="43"/>
     </row>
     <row r="3" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
@@ -1048,10 +1048,10 @@
       </c>
     </row>
     <row r="5" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A5" s="34" t="s">
+      <c r="A5" s="40" t="s">
         <v>64</v>
       </c>
-      <c r="B5" s="34"/>
+      <c r="B5" s="40"/>
     </row>
     <row r="6" spans="1:2" s="1" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A6" s="4" t="s">
@@ -1102,10 +1102,10 @@
       </c>
     </row>
     <row r="12" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A12" s="39" t="s">
+      <c r="A12" s="44" t="s">
         <v>67</v>
       </c>
-      <c r="B12" s="39"/>
+      <c r="B12" s="44"/>
     </row>
     <row r="13" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A13" s="20" t="s">
@@ -1140,10 +1140,10 @@
       </c>
     </row>
     <row r="17" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A17" s="40" t="s">
+      <c r="A17" s="45" t="s">
         <v>68</v>
       </c>
-      <c r="B17" s="40"/>
+      <c r="B17" s="45"/>
     </row>
     <row r="18" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A18" s="10" t="s">
@@ -1162,10 +1162,10 @@
       </c>
     </row>
     <row r="20" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A20" s="41" t="s">
+      <c r="A20" s="46" t="s">
         <v>69</v>
       </c>
-      <c r="B20" s="41"/>
+      <c r="B20" s="46"/>
     </row>
     <row r="21" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A21" s="12" t="s">
@@ -1208,10 +1208,10 @@
       </c>
     </row>
     <row r="26" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A26" s="42" t="s">
+      <c r="A26" s="47" t="s">
         <v>71</v>
       </c>
-      <c r="B26" s="42"/>
+      <c r="B26" s="47"/>
     </row>
     <row r="27" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A27" s="17" t="s">
@@ -1230,10 +1230,10 @@
       </c>
     </row>
     <row r="29" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
-      <c r="A29" s="43" t="s">
+      <c r="A29" s="48" t="s">
         <v>73</v>
       </c>
-      <c r="B29" s="43"/>
+      <c r="B29" s="48"/>
     </row>
     <row r="30" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A30" s="22" t="s">
@@ -1268,16 +1268,16 @@
       </c>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A34" s="35" t="s">
+      <c r="A34" s="41" t="s">
         <v>31</v>
       </c>
-      <c r="B34" s="37" t="s">
+      <c r="B34" s="36" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A35" s="36"/>
-      <c r="B35" s="37"/>
+      <c r="A35" s="42"/>
+      <c r="B35" s="36"/>
     </row>
     <row r="36" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A36" s="24" t="s">
@@ -1320,24 +1320,24 @@
       </c>
     </row>
     <row r="41" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A41" s="44" t="s">
+      <c r="A41" s="34" t="s">
         <v>76</v>
       </c>
-      <c r="B41" s="37" t="s">
+      <c r="B41" s="36" t="s">
         <v>77</v>
       </c>
     </row>
     <row r="42" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A42" s="45"/>
-      <c r="B42" s="37"/>
+      <c r="A42" s="35"/>
+      <c r="B42" s="36"/>
     </row>
     <row r="43" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A43" s="45"/>
-      <c r="B43" s="37"/>
+      <c r="A43" s="35"/>
+      <c r="B43" s="36"/>
     </row>
     <row r="44" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A44" s="45"/>
-      <c r="B44" s="37"/>
+      <c r="A44" s="35"/>
+      <c r="B44" s="36"/>
     </row>
     <row r="45" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A45" s="24" t="s">
@@ -1372,10 +1372,10 @@
       </c>
     </row>
     <row r="49" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A49" s="46" t="s">
+      <c r="A49" s="37" t="s">
         <v>75</v>
       </c>
-      <c r="B49" s="46"/>
+      <c r="B49" s="37"/>
     </row>
     <row r="50" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A50" s="25" t="s">
@@ -1434,10 +1434,10 @@
       </c>
     </row>
     <row r="57" spans="1:2" ht="18.5" x14ac:dyDescent="0.35">
-      <c r="A57" s="48" t="s">
+      <c r="A57" s="39" t="s">
         <v>70</v>
       </c>
-      <c r="B57" s="48"/>
+      <c r="B57" s="39"/>
     </row>
     <row r="58" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A58" s="14" t="s">
@@ -1524,10 +1524,10 @@
       </c>
     </row>
     <row r="69" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
-      <c r="A69" s="47" t="s">
+      <c r="A69" s="38" t="s">
         <v>108</v>
       </c>
-      <c r="B69" s="47"/>
+      <c r="B69" s="38"/>
     </row>
     <row r="70" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A70" s="32" t="s">
@@ -1547,11 +1547,6 @@
     </row>
   </sheetData>
   <mergeCells count="14">
-    <mergeCell ref="A41:A44"/>
-    <mergeCell ref="B41:B44"/>
-    <mergeCell ref="A49:B49"/>
-    <mergeCell ref="A69:B69"/>
-    <mergeCell ref="A57:B57"/>
     <mergeCell ref="A5:B5"/>
     <mergeCell ref="A34:A35"/>
     <mergeCell ref="B34:B35"/>
@@ -1561,6 +1556,11 @@
     <mergeCell ref="A20:B20"/>
     <mergeCell ref="A26:B26"/>
     <mergeCell ref="A29:B29"/>
+    <mergeCell ref="A41:A44"/>
+    <mergeCell ref="B41:B44"/>
+    <mergeCell ref="A49:B49"/>
+    <mergeCell ref="A69:B69"/>
+    <mergeCell ref="A57:B57"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
Reviewed 2 Problems 7/9/2026
</commit_message>
<xml_diff>
--- a/Code & Notes/Functions & Notes.xlsx
+++ b/Code & Notes/Functions & Notes.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\My Career\Courses\Web Development\Problem Solving\Code &amp; Notes\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\My Career\Problem Solving\Code &amp; Notes\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A6CE14E-42F3-4544-BA4C-E82C0969CC24}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B8BD2A2F-2C87-44C3-9B60-3D6FD1A4AA06}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="122" uniqueCount="118">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="116">
   <si>
     <t>Description</t>
   </si>
@@ -295,12 +295,6 @@
   </si>
   <si>
     <t>Find Nearest Square (prs)</t>
-  </si>
-  <si>
-    <t>/^[a-zA-Z]+$/.test(str[i])</t>
-  </si>
-  <si>
-    <t>Check If String Is Characters Only Not Numbers Or Special Characters</t>
   </si>
   <si>
     <t>Return text only and Remove special characters &amp; numbers &amp; spaces</t>
@@ -679,15 +673,42 @@
     <xf numFmtId="0" fontId="4" fillId="19" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="15" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="17" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -696,33 +717,6 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="15" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1010,7 +1004,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B71"/>
+  <dimension ref="A1:B70"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="91" customWidth="1"/>
@@ -1026,10 +1020,10 @@
       </c>
     </row>
     <row r="2" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A2" s="43" t="s">
+      <c r="A2" s="38" t="s">
         <v>63</v>
       </c>
-      <c r="B2" s="43"/>
+      <c r="B2" s="38"/>
     </row>
     <row r="3" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
@@ -1048,10 +1042,10 @@
       </c>
     </row>
     <row r="5" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A5" s="40" t="s">
+      <c r="A5" s="34" t="s">
         <v>64</v>
       </c>
-      <c r="B5" s="40"/>
+      <c r="B5" s="34"/>
     </row>
     <row r="6" spans="1:2" s="1" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A6" s="4" t="s">
@@ -1102,10 +1096,10 @@
       </c>
     </row>
     <row r="12" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A12" s="44" t="s">
+      <c r="A12" s="39" t="s">
         <v>67</v>
       </c>
-      <c r="B12" s="44"/>
+      <c r="B12" s="39"/>
     </row>
     <row r="13" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A13" s="20" t="s">
@@ -1140,10 +1134,10 @@
       </c>
     </row>
     <row r="17" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A17" s="45" t="s">
+      <c r="A17" s="40" t="s">
         <v>68</v>
       </c>
-      <c r="B17" s="45"/>
+      <c r="B17" s="40"/>
     </row>
     <row r="18" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A18" s="10" t="s">
@@ -1162,10 +1156,10 @@
       </c>
     </row>
     <row r="20" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A20" s="46" t="s">
+      <c r="A20" s="41" t="s">
         <v>69</v>
       </c>
-      <c r="B20" s="46"/>
+      <c r="B20" s="41"/>
     </row>
     <row r="21" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A21" s="12" t="s">
@@ -1201,17 +1195,17 @@
     </row>
     <row r="25" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A25" s="12" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="B25" s="28" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
     </row>
     <row r="26" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A26" s="47" t="s">
+      <c r="A26" s="42" t="s">
         <v>71</v>
       </c>
-      <c r="B26" s="47"/>
+      <c r="B26" s="42"/>
     </row>
     <row r="27" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A27" s="17" t="s">
@@ -1230,10 +1224,10 @@
       </c>
     </row>
     <row r="29" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
-      <c r="A29" s="48" t="s">
+      <c r="A29" s="43" t="s">
         <v>73</v>
       </c>
-      <c r="B29" s="48"/>
+      <c r="B29" s="43"/>
     </row>
     <row r="30" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A30" s="22" t="s">
@@ -1245,10 +1239,10 @@
     </row>
     <row r="31" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A31" s="23" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="B31" s="23" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
     </row>
     <row r="32" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
@@ -1268,16 +1262,16 @@
       </c>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A34" s="41" t="s">
+      <c r="A34" s="35" t="s">
         <v>31</v>
       </c>
-      <c r="B34" s="36" t="s">
+      <c r="B34" s="37" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A35" s="42"/>
-      <c r="B35" s="36"/>
+      <c r="A35" s="36"/>
+      <c r="B35" s="37"/>
     </row>
     <row r="36" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A36" s="24" t="s">
@@ -1289,7 +1283,7 @@
     </row>
     <row r="37" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A37" s="24" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="B37" s="23" t="s">
         <v>43</v>
@@ -1297,7 +1291,7 @@
     </row>
     <row r="38" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A38" s="24" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="B38" s="23" t="s">
         <v>44</v>
@@ -1320,24 +1314,24 @@
       </c>
     </row>
     <row r="41" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A41" s="34" t="s">
+      <c r="A41" s="44" t="s">
         <v>76</v>
       </c>
-      <c r="B41" s="36" t="s">
+      <c r="B41" s="37" t="s">
         <v>77</v>
       </c>
     </row>
     <row r="42" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A42" s="35"/>
-      <c r="B42" s="36"/>
+      <c r="A42" s="45"/>
+      <c r="B42" s="37"/>
     </row>
     <row r="43" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A43" s="35"/>
-      <c r="B43" s="36"/>
+      <c r="A43" s="45"/>
+      <c r="B43" s="37"/>
     </row>
     <row r="44" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A44" s="35"/>
-      <c r="B44" s="36"/>
+      <c r="A44" s="45"/>
+      <c r="B44" s="37"/>
     </row>
     <row r="45" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A45" s="24" t="s">
@@ -1357,25 +1351,25 @@
     </row>
     <row r="47" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A47" s="24" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="B47" s="22" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
     </row>
     <row r="48" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A48" s="24" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="B48" s="22" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
     </row>
     <row r="49" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A49" s="37" t="s">
+      <c r="A49" s="46" t="s">
         <v>75</v>
       </c>
-      <c r="B49" s="37"/>
+      <c r="B49" s="46"/>
     </row>
     <row r="50" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A50" s="25" t="s">
@@ -1406,38 +1400,38 @@
         <v>85</v>
       </c>
       <c r="B53" s="30" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
     </row>
     <row r="54" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A54" s="29" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="B54" s="30" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
     </row>
     <row r="55" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A55" s="29" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="B55" s="30" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
     </row>
     <row r="56" spans="1:2" ht="29" x14ac:dyDescent="0.35">
       <c r="A56" s="29" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="B56" s="30" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
     </row>
     <row r="57" spans="1:2" ht="18.5" x14ac:dyDescent="0.35">
-      <c r="A57" s="39" t="s">
+      <c r="A57" s="48" t="s">
         <v>70</v>
       </c>
-      <c r="B57" s="39"/>
+      <c r="B57" s="48"/>
     </row>
     <row r="58" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A58" s="14" t="s">
@@ -1452,7 +1446,7 @@
         <v>33</v>
       </c>
       <c r="B59" s="15" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
     </row>
     <row r="60" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
@@ -1472,7 +1466,7 @@
         <v>56</v>
       </c>
       <c r="B62" s="15" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
     </row>
     <row r="63" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
@@ -1492,61 +1486,58 @@
       </c>
     </row>
     <row r="65" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A65" s="16" t="s">
-        <v>88</v>
+      <c r="A65" s="31" t="s">
+        <v>97</v>
       </c>
       <c r="B65" s="15" t="s">
-        <v>89</v>
+        <v>98</v>
       </c>
     </row>
     <row r="66" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A66" s="31" t="s">
-        <v>99</v>
+      <c r="A66" s="16" t="s">
+        <v>104</v>
       </c>
       <c r="B66" s="15" t="s">
-        <v>100</v>
+        <v>105</v>
       </c>
     </row>
     <row r="67" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A67" s="16" t="s">
+        <v>110</v>
+      </c>
+      <c r="B67" s="15" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="68" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
+      <c r="A68" s="47" t="s">
         <v>106</v>
       </c>
-      <c r="B67" s="15" t="s">
+      <c r="B68" s="47"/>
+    </row>
+    <row r="69" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A69" s="32" t="s">
+        <v>108</v>
+      </c>
+      <c r="B69" s="33" t="s">
         <v>107</v>
       </c>
-    </row>
-    <row r="68" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A68" s="16" t="s">
-        <v>112</v>
-      </c>
-      <c r="B68" s="15" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="69" spans="1:2" ht="18.5" x14ac:dyDescent="0.45">
-      <c r="A69" s="38" t="s">
-        <v>108</v>
-      </c>
-      <c r="B69" s="38"/>
     </row>
     <row r="70" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A70" s="32" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="B70" s="33" t="s">
         <v>109</v>
       </c>
     </row>
-    <row r="71" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A71" s="32" t="s">
-        <v>110</v>
-      </c>
-      <c r="B71" s="33" t="s">
-        <v>111</v>
-      </c>
-    </row>
   </sheetData>
   <mergeCells count="14">
+    <mergeCell ref="A41:A44"/>
+    <mergeCell ref="B41:B44"/>
+    <mergeCell ref="A49:B49"/>
+    <mergeCell ref="A68:B68"/>
+    <mergeCell ref="A57:B57"/>
     <mergeCell ref="A5:B5"/>
     <mergeCell ref="A34:A35"/>
     <mergeCell ref="B34:B35"/>
@@ -1556,11 +1547,6 @@
     <mergeCell ref="A20:B20"/>
     <mergeCell ref="A26:B26"/>
     <mergeCell ref="A29:B29"/>
-    <mergeCell ref="A41:A44"/>
-    <mergeCell ref="B41:B44"/>
-    <mergeCell ref="A49:B49"/>
-    <mergeCell ref="A69:B69"/>
-    <mergeCell ref="A57:B57"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>